<commit_message>
Fix billing history discount column bug and migrate staff email to @roms.com
</commit_message>
<xml_diff>
--- a/bills_log.xlsx
+++ b/bills_log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -573,9 +573,125 @@
         <v>23.99</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>BILL-20260420-001</v>
+      </c>
+      <c r="B7" t="str">
+        <v>20/4/2026</v>
+      </c>
+      <c r="C7" t="str">
+        <v>4:45:45 pm</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Table 1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>wtest1</v>
+      </c>
+      <c r="F7" t="str">
+        <v>wather botel(½) x1 @₹5, Paneer Tikka x1 @₹11.5, Chicken Wings x1 @₹9.99, Garlic Bread x1 @₹4</v>
+      </c>
+      <c r="G7" t="str">
+        <v>30.49</v>
+      </c>
+      <c r="H7" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="I7" t="str">
+        <v>30.49</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>BILL-20260420-002</v>
+      </c>
+      <c r="B8" t="str">
+        <v>20/4/2026</v>
+      </c>
+      <c r="C8" t="str">
+        <v>4:49:46 pm</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Table 5</v>
+      </c>
+      <c r="E8" t="str">
+        <v>waitertest2</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Classic Burger x1 @₹12.99, Craft Beer x1 @₹5, Paneer Tikka x1 @₹11.5</v>
+      </c>
+      <c r="G8" t="str">
+        <v>29.49</v>
+      </c>
+      <c r="H8" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="I8" t="str">
+        <v>29.49</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>BILL-20260420-003</v>
+      </c>
+      <c r="B9" t="str">
+        <v>20/4/2026</v>
+      </c>
+      <c r="C9" t="str">
+        <v>4:49:52 pm</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Table 2</v>
+      </c>
+      <c r="E9" t="str">
+        <v>wtest1</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Garlic Bread x5 @₹4, Tiramisu x7 @₹6.5, Chicken Wings x4 @₹9.99</v>
+      </c>
+      <c r="G9" t="str">
+        <v>105.46</v>
+      </c>
+      <c r="H9" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="I9" t="str">
+        <v>105.46</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>BILL-20260420-004</v>
+      </c>
+      <c r="B10" t="str">
+        <v>20/4/2026</v>
+      </c>
+      <c r="C10" t="str">
+        <v>9:29:39 pm</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Table 6</v>
+      </c>
+      <c r="E10" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Classic Burger x1 @₹12.99, Pesto Pasta x1 @₹11, Caesar Salad x1 @₹8.5, Coke x1 @₹2.5, Craft Beer x1 @₹5</v>
+      </c>
+      <c r="G10" t="str">
+        <v>39.99</v>
+      </c>
+      <c r="H10" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="I10" t="str">
+        <v>39.99</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>